<commit_message>
changed model to calme3.2
</commit_message>
<xml_diff>
--- a/res/efficiency/pet-md/ollama-calme3.2-instruct-78b-Q4_K_S/2025-02-09_18-49-39/efficiency.xlsx
+++ b/res/efficiency/pet-md/ollama-calme3.2-instruct-78b-Q4_K_S/2025-02-09_18-49-39/efficiency.xlsx
@@ -1,17 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Felix\Documents\llm-process-generation\res\efficiency\pet-md\ollama-calme3.2-instruct-78b-Q4_K_S\2025-02-09_18-49-39\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BB33B6C-3113-45C1-BF82-7A7E9965B8BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="0" yWindow="1632" windowWidth="17280" windowHeight="10728" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Power_Stats" sheetId="1" r:id="rId1"/>
     <sheet name="Answer_Stats" sheetId="2" r:id="rId2"/>
     <sheet name="Error_Stats" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -90,8 +96,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -150,17 +156,25 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -198,7 +212,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -232,6 +246,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -266,9 +281,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -441,11 +457,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -456,7 +472,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -473,11 +489,14 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="4" width="14.109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -494,7 +513,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -511,7 +530,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -534,11 +553,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>19</v>
       </c>
@@ -546,7 +565,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>21</v>
       </c>

</xml_diff>

<commit_message>
changed model to AceInstruct Q4_K_S
</commit_message>
<xml_diff>
--- a/res/efficiency/pet-md/ollama-calme3.2-instruct-78b-Q4_K_S/2025-02-09_18-49-39/efficiency.xlsx
+++ b/res/efficiency/pet-md/ollama-calme3.2-instruct-78b-Q4_K_S/2025-02-09_18-49-39/efficiency.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Felix\Documents\llm-process-generation\res\efficiency\pet-md\ollama-calme3.2-instruct-78b-Q4_K_S\2025-02-09_18-49-39\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BB33B6C-3113-45C1-BF82-7A7E9965B8BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C32D653-BE71-4977-BA15-0DC0EFB239BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1632" windowWidth="17280" windowHeight="10728" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4752" yWindow="1044" windowWidth="17280" windowHeight="10728" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Power_Stats" sheetId="1" r:id="rId1"/>
@@ -460,6 +460,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.5546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -493,6 +498,7 @@
   <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="10.21875" bestFit="1" customWidth="1"/>
     <col min="2" max="4" width="14.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -556,6 +562,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.77734375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
added model name to file names for convenience
</commit_message>
<xml_diff>
--- a/res/efficiency/pet-md/ollama-calme3.2-instruct-78b-Q4_K_S/2025-02-09_18-49-39/efficiency.xlsx
+++ b/res/efficiency/pet-md/ollama-calme3.2-instruct-78b-Q4_K_S/2025-02-09_18-49-39/efficiency.xlsx
@@ -1,23 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28429"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Felix\Documents\llm-process-generation\res\efficiency\pet-md\ollama-calme3.2-instruct-78b-Q4_K_S\2025-02-09_18-49-39\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C32D653-BE71-4977-BA15-0DC0EFB239BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4752" yWindow="1044" windowWidth="17280" windowHeight="10728" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Power_Stats" sheetId="1" r:id="rId1"/>
     <sheet name="Answer_Stats" sheetId="2" r:id="rId2"/>
     <sheet name="Error_Stats" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -96,8 +90,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -156,25 +150,17 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -212,7 +198,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -246,7 +232,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -281,10 +266,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -457,16 +441,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.5546875" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -477,7 +456,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -494,15 +473,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="14.109375" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -519,7 +494,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -536,7 +511,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -559,15 +534,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.77734375" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>19</v>
       </c>
@@ -575,7 +546,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>21</v>
       </c>

</xml_diff>